<commit_message>
chore: commit pending local changes
</commit_message>
<xml_diff>
--- a/assessment/src/assessment_form/resources/assessment_application_materials.xlsx
+++ b/assessment/src/assessment_form/resources/assessment_application_materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WorkSpace\DocCollate\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\charlie\workspace\doccollate\assessment\src\assessment_form\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{733663EA-7A5C-4EEE-B8DC-7068940979B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE1CE31-8DD3-4219-AF8B-1F4F56E2BF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="第一步" sheetId="1" r:id="rId1"/>
@@ -502,6 +502,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -521,9 +524,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6108,28 +6108,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A7:F7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:F14"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6148,11 +6148,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="53.25" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -6238,10 +6238,10 @@
       <c r="K6" s="5"/>
     </row>
     <row r="7" spans="1:11" ht="20.25" customHeight="1">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="25"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="7"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -6253,10 +6253,10 @@
       <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11" ht="15">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="25"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
@@ -6270,8 +6270,8 @@
       <c r="K8" s="3"/>
     </row>
     <row r="9" spans="1:11" ht="15">
-      <c r="A9" s="29"/>
-      <c r="B9" s="30"/>
+      <c r="A9" s="30"/>
+      <c r="B9" s="31"/>
       <c r="C9" s="7" t="s">
         <v>9</v>
       </c>
@@ -6285,11 +6285,11 @@
       <c r="K9" s="3"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -6300,9 +6300,9 @@
       <c r="K10" s="3"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -6313,9 +6313,9 @@
       <c r="K11" s="3"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -6326,9 +6326,9 @@
       <c r="K12" s="3"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="27"/>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -6339,9 +6339,9 @@
       <c r="K13" s="3"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -6352,9 +6352,9 @@
       <c r="K14" s="3"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -6365,9 +6365,9 @@
       <c r="K15" s="3"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -6378,9 +6378,9 @@
       <c r="K16" s="3"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="27"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -6391,9 +6391,9 @@
       <c r="K17" s="3"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="27"/>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -6404,9 +6404,9 @@
       <c r="K18" s="3"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -6417,9 +6417,9 @@
       <c r="K19" s="3"/>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="27"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -6430,9 +6430,9 @@
       <c r="K20" s="3"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="27"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -6443,9 +6443,9 @@
       <c r="K21" s="3"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="27"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -6456,9 +6456,9 @@
       <c r="K22" s="3"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="27"/>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -8784,16 +8784,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A10:A23"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="B10:C23"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A10:A23"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="B10:C23"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>